<commit_message>
fix(specs-seed): split the Lonestar heading out of 26 09 61 2.8's General clause
The PDF-to-Word source ran "Automated Profile Fixture" into the General
clause's last sentence ("Permission to bid does not imply acceptance of the
manufacturer"), so the library's ENTERTAINMENT LUMINAIRES MOVING General
lost that sentence and the Lonestar product entry started with it. A
per-section split rule restores both; the converter also now reads only the
North HS section files in the source folder. Regenerated spec-library.json
(one article changed), the product-specs template and REVIEW-NOTES.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/specs-seed/northhs-2026-07-30/product-specs-template.xlsx
+++ b/docs/specs-seed/northhs-2026-07-30/product-specs-template.xlsx
@@ -2900,7 +2900,7 @@
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>ENTERTAINMENT LUMINAIRES MOVING</t>
+          <t>AUTOMATED PROFILE FIXTURE</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
@@ -2914,37 +2914,32 @@
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr"/>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>No heading in the source — Spec Title taken from the article.</t>
-        </is>
-      </c>
+      <c r="H41" s="4" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
-          <t>Permission to bid does not imply acceptance of the manufacturer Automated Profile Fixture
-  Basis of Design: Lonestar as manufactured by ETC Inc.
-  Standards Compliance:
-    Listed: UL 1573, and CE Certification
-  Array:
-    Ultra-Bright 7000K
-  Features:
-    Four Plane Shutter System
-    Nine Rotating Interchangeable Gobos
-    CYM Subtractive Color Mixing
-    Ten Interchangeable Colors
-      Red, blue, green, yellow, orange, purple, TM-30 filter, lavender, half CTO, full CTO, and dark blue
-    Pan Tilt and Zoom
-      Pan 540 Degrees, 360 movement in 2.3s
-      Tilt 270 Degrees, 180 movement in 1.26s
-      Zoom 3.8-55 Degrees
-  Control:
-    Input Method:
-      DMX-512 via 5-Pin. Protocols: DMX512, RDM.
-      Ethernet via RJ45, Protocols: SACN, ArtNet
-  Electrical:
-    Input Method: powerCON True1 TOP in and thru.
-    Fixtures per Circuit:
-      Two</t>
+          <t>Basis of Design: Lonestar as manufactured by ETC Inc.
+Standards Compliance:
+  Listed: UL 1573, and CE Certification
+Array:
+  Ultra-Bright 7000K
+Features:
+  Four Plane Shutter System
+  Nine Rotating Interchangeable Gobos
+  CYM Subtractive Color Mixing
+  Ten Interchangeable Colors
+    Red, blue, green, yellow, orange, purple, TM-30 filter, lavender, half CTO, full CTO, and dark blue
+  Pan Tilt and Zoom
+    Pan 540 Degrees, 360 movement in 2.3s
+    Tilt 270 Degrees, 180 movement in 1.26s
+    Zoom 3.8-55 Degrees
+Control:
+  Input Method:
+    DMX-512 via 5-Pin. Protocols: DMX512, RDM.
+    Ethernet via RJ45, Protocols: SACN, ArtNet
+Electrical:
+  Input Method: powerCON True1 TOP in and thru.
+  Fixtures per Circuit:
+    Two</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">

</xml_diff>